<commit_message>
update graph plot legend
</commit_message>
<xml_diff>
--- a/temp_table.xlsx
+++ b/temp_table.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usi365-my.sharepoint.com/personal/fenogd_usi_ch/Documents/PC/Desktop/USI_Locale/Federated-C2BM/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dariofenoglio/Desktop/Federated-C2BM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{CF1EF59A-8F47-0840-BC75-97268760C1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8894E5C-AAA0-8748-A601-FA969C97372E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0209054-CF73-D743-B14F-40084AE0566F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27900" yWindow="5380" windowWidth="29000" windowHeight="18960" xr2:uid="{8C3DF6BF-8DDD-F446-8EAC-CCE1EEDA313F}"/>
+    <workbookView xWindow="27900" yWindow="5380" windowWidth="29000" windowHeight="18960" activeTab="5" xr2:uid="{8C3DF6BF-8DDD-F446-8EAC-CCE1EEDA313F}"/>
   </bookViews>
   <sheets>
     <sheet name="Asia" sheetId="1" r:id="rId1"/>
@@ -76,13 +76,13 @@
     <t>Asia</t>
   </si>
   <si>
-    <t>TFL</t>
-  </si>
-  <si>
     <t>Loc.</t>
   </si>
   <si>
-    <t>Ours</t>
+    <t>F-CMs (Ours)</t>
+  </si>
+  <si>
+    <t>S-F-CMs</t>
   </si>
 </sst>
 </file>
@@ -619,33 +619,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -677,6 +650,33 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1131,130 +1131,130 @@
       <c r="T12" s="6"/>
     </row>
     <row r="13" spans="4:24" x14ac:dyDescent="0.2">
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="33"/>
-      <c r="I13" s="33"/>
-      <c r="J13" s="33"/>
-      <c r="K13" s="33"/>
-      <c r="L13" s="33"/>
-      <c r="M13" s="33"/>
-      <c r="N13" s="33"/>
-      <c r="O13" s="33"/>
-      <c r="P13" s="33"/>
-      <c r="Q13" s="33"/>
-      <c r="R13" s="33"/>
-      <c r="S13" s="33"/>
-      <c r="T13" s="33"/>
-      <c r="U13" s="33"/>
-      <c r="V13" s="33"/>
-      <c r="W13" s="33"/>
-      <c r="X13" s="34"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="44"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="44"/>
+      <c r="R13" s="44"/>
+      <c r="S13" s="44"/>
+      <c r="T13" s="44"/>
+      <c r="U13" s="44"/>
+      <c r="V13" s="44"/>
+      <c r="W13" s="44"/>
+      <c r="X13" s="45"/>
     </row>
     <row r="14" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="G14" s="35"/>
-      <c r="H14" s="36"/>
-      <c r="I14" s="36"/>
-      <c r="J14" s="36"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="36"/>
-      <c r="O14" s="36"/>
-      <c r="P14" s="36"/>
-      <c r="Q14" s="36"/>
-      <c r="R14" s="36"/>
-      <c r="S14" s="36"/>
-      <c r="T14" s="36"/>
-      <c r="U14" s="36"/>
-      <c r="V14" s="36"/>
-      <c r="W14" s="36"/>
-      <c r="X14" s="37"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="47"/>
+      <c r="L14" s="47"/>
+      <c r="M14" s="47"/>
+      <c r="N14" s="47"/>
+      <c r="O14" s="47"/>
+      <c r="P14" s="47"/>
+      <c r="Q14" s="47"/>
+      <c r="R14" s="47"/>
+      <c r="S14" s="47"/>
+      <c r="T14" s="47"/>
+      <c r="U14" s="47"/>
+      <c r="V14" s="47"/>
+      <c r="W14" s="47"/>
+      <c r="X14" s="48"/>
     </row>
     <row r="15" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="E15" s="39"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="38">
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="49">
         <v>0.1</v>
       </c>
-      <c r="H15" s="40"/>
-      <c r="I15" s="38">
+      <c r="H15" s="51"/>
+      <c r="I15" s="49">
         <v>0.2</v>
       </c>
-      <c r="J15" s="40"/>
-      <c r="K15" s="38">
+      <c r="J15" s="51"/>
+      <c r="K15" s="49">
         <v>0.3</v>
       </c>
-      <c r="L15" s="40"/>
-      <c r="M15" s="38">
+      <c r="L15" s="51"/>
+      <c r="M15" s="49">
         <v>0.4</v>
       </c>
-      <c r="N15" s="40"/>
-      <c r="O15" s="38">
+      <c r="N15" s="51"/>
+      <c r="O15" s="49">
         <v>0.5</v>
       </c>
-      <c r="P15" s="40"/>
-      <c r="Q15" s="38">
+      <c r="P15" s="51"/>
+      <c r="Q15" s="49">
         <v>0.6</v>
       </c>
-      <c r="R15" s="40"/>
-      <c r="S15" s="38">
+      <c r="R15" s="51"/>
+      <c r="S15" s="49">
         <v>0.7</v>
       </c>
-      <c r="T15" s="40"/>
-      <c r="U15" s="38">
+      <c r="T15" s="51"/>
+      <c r="U15" s="49">
         <v>0.8</v>
       </c>
-      <c r="V15" s="40"/>
-      <c r="W15" s="38">
+      <c r="V15" s="51"/>
+      <c r="W15" s="49">
         <v>0.9</v>
       </c>
-      <c r="X15" s="40"/>
+      <c r="X15" s="51"/>
     </row>
     <row r="16" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D16" s="8"/>
       <c r="E16" s="27"/>
       <c r="F16" s="9"/>
-      <c r="G16" s="41" t="s">
+      <c r="G16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="H16" s="42"/>
-      <c r="I16" s="41" t="s">
+      <c r="H16" s="33"/>
+      <c r="I16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="J16" s="42"/>
-      <c r="K16" s="41" t="s">
+      <c r="J16" s="33"/>
+      <c r="K16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="L16" s="51"/>
-      <c r="M16" s="41" t="s">
+      <c r="L16" s="42"/>
+      <c r="M16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="N16" s="42"/>
-      <c r="O16" s="41" t="s">
+      <c r="N16" s="33"/>
+      <c r="O16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="41" t="s">
+      <c r="P16" s="33"/>
+      <c r="Q16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="R16" s="42"/>
-      <c r="S16" s="41" t="s">
+      <c r="R16" s="33"/>
+      <c r="S16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="T16" s="42"/>
-      <c r="U16" s="43" t="s">
+      <c r="T16" s="33"/>
+      <c r="U16" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="V16" s="44"/>
-      <c r="W16" s="43" t="s">
+      <c r="V16" s="35"/>
+      <c r="W16" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="X16" s="44"/>
+      <c r="X16" s="35"/>
     </row>
     <row r="17" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D17" s="10"/>
@@ -1316,75 +1316,75 @@
       </c>
     </row>
     <row r="18" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="45" t="s">
+      <c r="D18" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="48">
+      <c r="E18" s="39">
         <v>0.3</v>
       </c>
       <c r="F18" s="29" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="15">
+        <v>0</v>
+      </c>
+      <c r="H18" s="3">
+        <v>0</v>
+      </c>
+      <c r="I18" s="4">
+        <v>0</v>
+      </c>
+      <c r="J18" s="5">
+        <v>0</v>
+      </c>
+      <c r="K18" s="4">
+        <v>0</v>
+      </c>
+      <c r="L18" s="16">
+        <v>0</v>
+      </c>
+      <c r="M18" s="4">
+        <v>0</v>
+      </c>
+      <c r="N18" s="5">
+        <v>0</v>
+      </c>
+      <c r="O18" s="4">
+        <v>0</v>
+      </c>
+      <c r="P18" s="5">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="4">
+        <v>0</v>
+      </c>
+      <c r="R18" s="5">
+        <v>0</v>
+      </c>
+      <c r="S18" s="4">
+        <v>0</v>
+      </c>
+      <c r="T18" s="5">
+        <v>0</v>
+      </c>
+      <c r="U18" s="4">
+        <v>0</v>
+      </c>
+      <c r="V18" s="5">
+        <v>0</v>
+      </c>
+      <c r="W18" s="15">
+        <v>0</v>
+      </c>
+      <c r="X18" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="D19" s="37"/>
+      <c r="E19" s="40"/>
+      <c r="F19" s="29" t="s">
         <v>13</v>
-      </c>
-      <c r="G18" s="15">
-        <v>0</v>
-      </c>
-      <c r="H18" s="3">
-        <v>0</v>
-      </c>
-      <c r="I18" s="4">
-        <v>0</v>
-      </c>
-      <c r="J18" s="5">
-        <v>0</v>
-      </c>
-      <c r="K18" s="4">
-        <v>0</v>
-      </c>
-      <c r="L18" s="16">
-        <v>0</v>
-      </c>
-      <c r="M18" s="4">
-        <v>0</v>
-      </c>
-      <c r="N18" s="5">
-        <v>0</v>
-      </c>
-      <c r="O18" s="4">
-        <v>0</v>
-      </c>
-      <c r="P18" s="5">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="4">
-        <v>0</v>
-      </c>
-      <c r="R18" s="5">
-        <v>0</v>
-      </c>
-      <c r="S18" s="4">
-        <v>0</v>
-      </c>
-      <c r="T18" s="5">
-        <v>0</v>
-      </c>
-      <c r="U18" s="4">
-        <v>0</v>
-      </c>
-      <c r="V18" s="5">
-        <v>0</v>
-      </c>
-      <c r="W18" s="15">
-        <v>0</v>
-      </c>
-      <c r="X18" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="46"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="29" t="s">
-        <v>11</v>
       </c>
       <c r="G19" s="17">
         <v>4.8</v>
@@ -1442,10 +1442,10 @@
       </c>
     </row>
     <row r="20" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D20" s="46"/>
-      <c r="E20" s="50"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="41"/>
       <c r="F20" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G20" s="21">
         <v>4.3659999999999997</v>
@@ -1503,12 +1503,12 @@
       </c>
     </row>
     <row r="21" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D21" s="46"/>
-      <c r="E21" s="48">
+      <c r="D21" s="37"/>
+      <c r="E21" s="39">
         <v>0.6</v>
       </c>
       <c r="F21" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G21" s="30">
         <v>0</v>
@@ -1566,10 +1566,10 @@
       </c>
     </row>
     <row r="22" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D22" s="46"/>
-      <c r="E22" s="49"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="40"/>
       <c r="F22" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G22" s="30">
         <v>4.8</v>
@@ -1627,10 +1627,10 @@
       </c>
     </row>
     <row r="23" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="46"/>
-      <c r="E23" s="50"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="41"/>
       <c r="F23" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G23" s="31">
         <v>4.6529999999999996</v>
@@ -1688,12 +1688,12 @@
       </c>
     </row>
     <row r="24" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D24" s="46"/>
-      <c r="E24" s="48">
+      <c r="D24" s="37"/>
+      <c r="E24" s="39">
         <v>0.9</v>
       </c>
       <c r="F24" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G24" s="30">
         <v>0</v>
@@ -1751,10 +1751,10 @@
       </c>
     </row>
     <row r="25" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D25" s="46"/>
-      <c r="E25" s="49"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="40"/>
       <c r="F25" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G25" s="30">
         <v>4.8</v>
@@ -1812,10 +1812,10 @@
       </c>
     </row>
     <row r="26" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D26" s="47"/>
-      <c r="E26" s="50"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="41"/>
       <c r="F26" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G26" s="31">
         <v>4.8949999999999996</v>
@@ -1950,6 +1950,17 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="G13:X14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="U15:V15"/>
+    <mergeCell ref="W15:X15"/>
+    <mergeCell ref="S15:T15"/>
     <mergeCell ref="Q16:R16"/>
     <mergeCell ref="S16:T16"/>
     <mergeCell ref="U16:V16"/>
@@ -1963,17 +1974,6 @@
     <mergeCell ref="K16:L16"/>
     <mergeCell ref="M16:N16"/>
     <mergeCell ref="O16:P16"/>
-    <mergeCell ref="G13:X14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="U15:V15"/>
-    <mergeCell ref="W15:X15"/>
-    <mergeCell ref="S15:T15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1986,130 +1986,130 @@
   <sheetData>
     <row r="12" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="4:24" x14ac:dyDescent="0.2">
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="H13" s="33"/>
-      <c r="I13" s="33"/>
-      <c r="J13" s="33"/>
-      <c r="K13" s="33"/>
-      <c r="L13" s="33"/>
-      <c r="M13" s="33"/>
-      <c r="N13" s="33"/>
-      <c r="O13" s="33"/>
-      <c r="P13" s="33"/>
-      <c r="Q13" s="33"/>
-      <c r="R13" s="33"/>
-      <c r="S13" s="33"/>
-      <c r="T13" s="33"/>
-      <c r="U13" s="33"/>
-      <c r="V13" s="33"/>
-      <c r="W13" s="33"/>
-      <c r="X13" s="34"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="44"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="44"/>
+      <c r="R13" s="44"/>
+      <c r="S13" s="44"/>
+      <c r="T13" s="44"/>
+      <c r="U13" s="44"/>
+      <c r="V13" s="44"/>
+      <c r="W13" s="44"/>
+      <c r="X13" s="45"/>
     </row>
     <row r="14" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="G14" s="35"/>
-      <c r="H14" s="36"/>
-      <c r="I14" s="36"/>
-      <c r="J14" s="36"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="36"/>
-      <c r="O14" s="36"/>
-      <c r="P14" s="36"/>
-      <c r="Q14" s="36"/>
-      <c r="R14" s="36"/>
-      <c r="S14" s="36"/>
-      <c r="T14" s="36"/>
-      <c r="U14" s="36"/>
-      <c r="V14" s="36"/>
-      <c r="W14" s="36"/>
-      <c r="X14" s="37"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="47"/>
+      <c r="L14" s="47"/>
+      <c r="M14" s="47"/>
+      <c r="N14" s="47"/>
+      <c r="O14" s="47"/>
+      <c r="P14" s="47"/>
+      <c r="Q14" s="47"/>
+      <c r="R14" s="47"/>
+      <c r="S14" s="47"/>
+      <c r="T14" s="47"/>
+      <c r="U14" s="47"/>
+      <c r="V14" s="47"/>
+      <c r="W14" s="47"/>
+      <c r="X14" s="48"/>
     </row>
     <row r="15" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="E15" s="39"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="38">
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="49">
         <v>0.1</v>
       </c>
-      <c r="H15" s="40"/>
-      <c r="I15" s="38">
+      <c r="H15" s="51"/>
+      <c r="I15" s="49">
         <v>0.2</v>
       </c>
-      <c r="J15" s="40"/>
-      <c r="K15" s="38">
+      <c r="J15" s="51"/>
+      <c r="K15" s="49">
         <v>0.3</v>
       </c>
-      <c r="L15" s="40"/>
-      <c r="M15" s="38">
+      <c r="L15" s="51"/>
+      <c r="M15" s="49">
         <v>0.4</v>
       </c>
-      <c r="N15" s="40"/>
-      <c r="O15" s="38">
+      <c r="N15" s="51"/>
+      <c r="O15" s="49">
         <v>0.5</v>
       </c>
-      <c r="P15" s="40"/>
-      <c r="Q15" s="38">
+      <c r="P15" s="51"/>
+      <c r="Q15" s="49">
         <v>0.6</v>
       </c>
-      <c r="R15" s="40"/>
-      <c r="S15" s="38">
+      <c r="R15" s="51"/>
+      <c r="S15" s="49">
         <v>0.7</v>
       </c>
-      <c r="T15" s="40"/>
-      <c r="U15" s="38">
+      <c r="T15" s="51"/>
+      <c r="U15" s="49">
         <v>0.8</v>
       </c>
-      <c r="V15" s="40"/>
-      <c r="W15" s="38">
+      <c r="V15" s="51"/>
+      <c r="W15" s="49">
         <v>0.9</v>
       </c>
-      <c r="X15" s="40"/>
+      <c r="X15" s="51"/>
     </row>
     <row r="16" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D16" s="8"/>
       <c r="E16" s="27"/>
       <c r="F16" s="9"/>
-      <c r="G16" s="41" t="s">
+      <c r="G16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="H16" s="42"/>
-      <c r="I16" s="41" t="s">
+      <c r="H16" s="33"/>
+      <c r="I16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="J16" s="42"/>
-      <c r="K16" s="41" t="s">
+      <c r="J16" s="33"/>
+      <c r="K16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="L16" s="51"/>
-      <c r="M16" s="41" t="s">
+      <c r="L16" s="42"/>
+      <c r="M16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="N16" s="42"/>
-      <c r="O16" s="41" t="s">
+      <c r="N16" s="33"/>
+      <c r="O16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="41" t="s">
+      <c r="P16" s="33"/>
+      <c r="Q16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="R16" s="42"/>
-      <c r="S16" s="41" t="s">
+      <c r="R16" s="33"/>
+      <c r="S16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="T16" s="42"/>
-      <c r="U16" s="43" t="s">
+      <c r="T16" s="33"/>
+      <c r="U16" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="V16" s="44"/>
-      <c r="W16" s="43" t="s">
+      <c r="V16" s="35"/>
+      <c r="W16" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="X16" s="44"/>
+      <c r="X16" s="35"/>
     </row>
     <row r="17" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D17" s="10"/>
@@ -2171,14 +2171,14 @@
       </c>
     </row>
     <row r="18" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="45" t="s">
+      <c r="D18" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="48">
+      <c r="E18" s="39">
         <v>0.3</v>
       </c>
       <c r="F18" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G18" s="15">
         <v>0.8</v>
@@ -2236,10 +2236,10 @@
       </c>
     </row>
     <row r="19" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="46"/>
-      <c r="E19" s="49"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="40"/>
       <c r="F19" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G19" s="17">
         <v>11</v>
@@ -2297,10 +2297,10 @@
       </c>
     </row>
     <row r="20" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D20" s="46"/>
-      <c r="E20" s="50"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="41"/>
       <c r="F20" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G20" s="21">
         <v>11.53</v>
@@ -2358,12 +2358,12 @@
       </c>
     </row>
     <row r="21" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D21" s="46"/>
-      <c r="E21" s="48">
+      <c r="D21" s="37"/>
+      <c r="E21" s="39">
         <v>0.6</v>
       </c>
       <c r="F21" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G21" s="30">
         <v>0.8</v>
@@ -2421,10 +2421,10 @@
       </c>
     </row>
     <row r="22" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D22" s="46"/>
-      <c r="E22" s="49"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="40"/>
       <c r="F22" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G22" s="30">
         <v>11</v>
@@ -2482,10 +2482,10 @@
       </c>
     </row>
     <row r="23" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="46"/>
-      <c r="E23" s="50"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="41"/>
       <c r="F23" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G23" s="31">
         <v>11.87</v>
@@ -2543,12 +2543,12 @@
       </c>
     </row>
     <row r="24" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D24" s="46"/>
-      <c r="E24" s="48">
+      <c r="D24" s="37"/>
+      <c r="E24" s="39">
         <v>0.9</v>
       </c>
       <c r="F24" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G24" s="30">
         <v>0.8</v>
@@ -2606,10 +2606,10 @@
       </c>
     </row>
     <row r="25" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D25" s="46"/>
-      <c r="E25" s="49"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="40"/>
       <c r="F25" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G25" s="30">
         <v>11</v>
@@ -2667,10 +2667,10 @@
       </c>
     </row>
     <row r="26" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D26" s="47"/>
-      <c r="E26" s="50"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="41"/>
       <c r="F26" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G26" s="31">
         <v>12.154</v>
@@ -2729,16 +2729,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="G13:X14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="S15:T15"/>
-    <mergeCell ref="U15:V15"/>
     <mergeCell ref="D18:D26"/>
     <mergeCell ref="E18:E20"/>
     <mergeCell ref="E21:E23"/>
@@ -2753,6 +2743,16 @@
     <mergeCell ref="S16:T16"/>
     <mergeCell ref="U16:V16"/>
     <mergeCell ref="W16:X16"/>
+    <mergeCell ref="G13:X14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="S15:T15"/>
+    <mergeCell ref="U15:V15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2765,130 +2765,130 @@
   <sheetData>
     <row r="12" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="4:24" x14ac:dyDescent="0.2">
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="H13" s="33"/>
-      <c r="I13" s="33"/>
-      <c r="J13" s="33"/>
-      <c r="K13" s="33"/>
-      <c r="L13" s="33"/>
-      <c r="M13" s="33"/>
-      <c r="N13" s="33"/>
-      <c r="O13" s="33"/>
-      <c r="P13" s="33"/>
-      <c r="Q13" s="33"/>
-      <c r="R13" s="33"/>
-      <c r="S13" s="33"/>
-      <c r="T13" s="33"/>
-      <c r="U13" s="33"/>
-      <c r="V13" s="33"/>
-      <c r="W13" s="33"/>
-      <c r="X13" s="34"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="44"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="44"/>
+      <c r="R13" s="44"/>
+      <c r="S13" s="44"/>
+      <c r="T13" s="44"/>
+      <c r="U13" s="44"/>
+      <c r="V13" s="44"/>
+      <c r="W13" s="44"/>
+      <c r="X13" s="45"/>
     </row>
     <row r="14" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="G14" s="35"/>
-      <c r="H14" s="36"/>
-      <c r="I14" s="36"/>
-      <c r="J14" s="36"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="36"/>
-      <c r="O14" s="36"/>
-      <c r="P14" s="36"/>
-      <c r="Q14" s="36"/>
-      <c r="R14" s="36"/>
-      <c r="S14" s="36"/>
-      <c r="T14" s="36"/>
-      <c r="U14" s="36"/>
-      <c r="V14" s="36"/>
-      <c r="W14" s="36"/>
-      <c r="X14" s="37"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="47"/>
+      <c r="L14" s="47"/>
+      <c r="M14" s="47"/>
+      <c r="N14" s="47"/>
+      <c r="O14" s="47"/>
+      <c r="P14" s="47"/>
+      <c r="Q14" s="47"/>
+      <c r="R14" s="47"/>
+      <c r="S14" s="47"/>
+      <c r="T14" s="47"/>
+      <c r="U14" s="47"/>
+      <c r="V14" s="47"/>
+      <c r="W14" s="47"/>
+      <c r="X14" s="48"/>
     </row>
     <row r="15" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="E15" s="39"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="38">
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="49">
         <v>0.1</v>
       </c>
-      <c r="H15" s="40"/>
-      <c r="I15" s="38">
+      <c r="H15" s="51"/>
+      <c r="I15" s="49">
         <v>0.2</v>
       </c>
-      <c r="J15" s="40"/>
-      <c r="K15" s="38">
+      <c r="J15" s="51"/>
+      <c r="K15" s="49">
         <v>0.3</v>
       </c>
-      <c r="L15" s="40"/>
-      <c r="M15" s="38">
+      <c r="L15" s="51"/>
+      <c r="M15" s="49">
         <v>0.4</v>
       </c>
-      <c r="N15" s="40"/>
-      <c r="O15" s="38">
+      <c r="N15" s="51"/>
+      <c r="O15" s="49">
         <v>0.5</v>
       </c>
-      <c r="P15" s="40"/>
-      <c r="Q15" s="38">
+      <c r="P15" s="51"/>
+      <c r="Q15" s="49">
         <v>0.6</v>
       </c>
-      <c r="R15" s="40"/>
-      <c r="S15" s="38">
+      <c r="R15" s="51"/>
+      <c r="S15" s="49">
         <v>0.7</v>
       </c>
-      <c r="T15" s="40"/>
-      <c r="U15" s="38">
+      <c r="T15" s="51"/>
+      <c r="U15" s="49">
         <v>0.8</v>
       </c>
-      <c r="V15" s="40"/>
-      <c r="W15" s="38">
+      <c r="V15" s="51"/>
+      <c r="W15" s="49">
         <v>0.9</v>
       </c>
-      <c r="X15" s="40"/>
+      <c r="X15" s="51"/>
     </row>
     <row r="16" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D16" s="8"/>
       <c r="E16" s="27"/>
       <c r="F16" s="9"/>
-      <c r="G16" s="41" t="s">
+      <c r="G16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="H16" s="42"/>
-      <c r="I16" s="41" t="s">
+      <c r="H16" s="33"/>
+      <c r="I16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="J16" s="42"/>
-      <c r="K16" s="41" t="s">
+      <c r="J16" s="33"/>
+      <c r="K16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="L16" s="51"/>
-      <c r="M16" s="41" t="s">
+      <c r="L16" s="42"/>
+      <c r="M16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="N16" s="42"/>
-      <c r="O16" s="41" t="s">
+      <c r="N16" s="33"/>
+      <c r="O16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="41" t="s">
+      <c r="P16" s="33"/>
+      <c r="Q16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="R16" s="42"/>
-      <c r="S16" s="41" t="s">
+      <c r="R16" s="33"/>
+      <c r="S16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="T16" s="42"/>
-      <c r="U16" s="43" t="s">
+      <c r="T16" s="33"/>
+      <c r="U16" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="V16" s="44"/>
-      <c r="W16" s="43" t="s">
+      <c r="V16" s="35"/>
+      <c r="W16" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="X16" s="44"/>
+      <c r="X16" s="35"/>
     </row>
     <row r="17" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D17" s="10"/>
@@ -2950,14 +2950,14 @@
       </c>
     </row>
     <row r="18" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="45" t="s">
+      <c r="D18" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="48">
+      <c r="E18" s="39">
         <v>0.3</v>
       </c>
       <c r="F18" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G18" s="15">
         <v>2.2000000000000002</v>
@@ -3015,10 +3015,10 @@
       </c>
     </row>
     <row r="19" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="46"/>
-      <c r="E19" s="49"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="40"/>
       <c r="F19" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G19" s="17">
         <v>21.4</v>
@@ -3076,10 +3076,10 @@
       </c>
     </row>
     <row r="20" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D20" s="46"/>
-      <c r="E20" s="50"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="41"/>
       <c r="F20" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G20" s="21">
         <v>33.658000000000001</v>
@@ -3137,12 +3137,12 @@
       </c>
     </row>
     <row r="21" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D21" s="46"/>
-      <c r="E21" s="48">
+      <c r="D21" s="37"/>
+      <c r="E21" s="39">
         <v>0.6</v>
       </c>
       <c r="F21" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G21" s="30">
         <v>2.2000000000000002</v>
@@ -3200,10 +3200,10 @@
       </c>
     </row>
     <row r="22" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D22" s="46"/>
-      <c r="E22" s="49"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="40"/>
       <c r="F22" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G22" s="30">
         <v>21.4</v>
@@ -3261,10 +3261,10 @@
       </c>
     </row>
     <row r="23" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="46"/>
-      <c r="E23" s="50"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="41"/>
       <c r="F23" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G23" s="31">
         <v>35.469000000000001</v>
@@ -3322,12 +3322,12 @@
       </c>
     </row>
     <row r="24" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D24" s="46"/>
-      <c r="E24" s="48">
+      <c r="D24" s="37"/>
+      <c r="E24" s="39">
         <v>0.9</v>
       </c>
       <c r="F24" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G24" s="30">
         <v>2.2000000000000002</v>
@@ -3385,10 +3385,10 @@
       </c>
     </row>
     <row r="25" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D25" s="46"/>
-      <c r="E25" s="49"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="40"/>
       <c r="F25" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G25" s="30">
         <v>21.4</v>
@@ -3446,10 +3446,10 @@
       </c>
     </row>
     <row r="26" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D26" s="47"/>
-      <c r="E26" s="50"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="41"/>
       <c r="F26" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G26" s="31">
         <v>37.119</v>
@@ -3508,16 +3508,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="G13:X14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="S15:T15"/>
-    <mergeCell ref="U15:V15"/>
     <mergeCell ref="D18:D26"/>
     <mergeCell ref="E18:E20"/>
     <mergeCell ref="E21:E23"/>
@@ -3532,6 +3522,16 @@
     <mergeCell ref="S16:T16"/>
     <mergeCell ref="U16:V16"/>
     <mergeCell ref="W16:X16"/>
+    <mergeCell ref="G13:X14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="S15:T15"/>
+    <mergeCell ref="U15:V15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3544,130 +3544,130 @@
   <sheetData>
     <row r="12" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="4:24" x14ac:dyDescent="0.2">
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="H13" s="33"/>
-      <c r="I13" s="33"/>
-      <c r="J13" s="33"/>
-      <c r="K13" s="33"/>
-      <c r="L13" s="33"/>
-      <c r="M13" s="33"/>
-      <c r="N13" s="33"/>
-      <c r="O13" s="33"/>
-      <c r="P13" s="33"/>
-      <c r="Q13" s="33"/>
-      <c r="R13" s="33"/>
-      <c r="S13" s="33"/>
-      <c r="T13" s="33"/>
-      <c r="U13" s="33"/>
-      <c r="V13" s="33"/>
-      <c r="W13" s="33"/>
-      <c r="X13" s="34"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="44"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="44"/>
+      <c r="R13" s="44"/>
+      <c r="S13" s="44"/>
+      <c r="T13" s="44"/>
+      <c r="U13" s="44"/>
+      <c r="V13" s="44"/>
+      <c r="W13" s="44"/>
+      <c r="X13" s="45"/>
     </row>
     <row r="14" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="G14" s="35"/>
-      <c r="H14" s="36"/>
-      <c r="I14" s="36"/>
-      <c r="J14" s="36"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="36"/>
-      <c r="O14" s="36"/>
-      <c r="P14" s="36"/>
-      <c r="Q14" s="36"/>
-      <c r="R14" s="36"/>
-      <c r="S14" s="36"/>
-      <c r="T14" s="36"/>
-      <c r="U14" s="36"/>
-      <c r="V14" s="36"/>
-      <c r="W14" s="36"/>
-      <c r="X14" s="37"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="47"/>
+      <c r="L14" s="47"/>
+      <c r="M14" s="47"/>
+      <c r="N14" s="47"/>
+      <c r="O14" s="47"/>
+      <c r="P14" s="47"/>
+      <c r="Q14" s="47"/>
+      <c r="R14" s="47"/>
+      <c r="S14" s="47"/>
+      <c r="T14" s="47"/>
+      <c r="U14" s="47"/>
+      <c r="V14" s="47"/>
+      <c r="W14" s="47"/>
+      <c r="X14" s="48"/>
     </row>
     <row r="15" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="E15" s="39"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="38">
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="49">
         <v>0.1</v>
       </c>
-      <c r="H15" s="40"/>
-      <c r="I15" s="38">
+      <c r="H15" s="51"/>
+      <c r="I15" s="49">
         <v>0.2</v>
       </c>
-      <c r="J15" s="40"/>
-      <c r="K15" s="38">
+      <c r="J15" s="51"/>
+      <c r="K15" s="49">
         <v>0.3</v>
       </c>
-      <c r="L15" s="40"/>
-      <c r="M15" s="38">
+      <c r="L15" s="51"/>
+      <c r="M15" s="49">
         <v>0.4</v>
       </c>
-      <c r="N15" s="40"/>
-      <c r="O15" s="38">
+      <c r="N15" s="51"/>
+      <c r="O15" s="49">
         <v>0.5</v>
       </c>
-      <c r="P15" s="40"/>
-      <c r="Q15" s="38">
+      <c r="P15" s="51"/>
+      <c r="Q15" s="49">
         <v>0.6</v>
       </c>
-      <c r="R15" s="40"/>
-      <c r="S15" s="38">
+      <c r="R15" s="51"/>
+      <c r="S15" s="49">
         <v>0.7</v>
       </c>
-      <c r="T15" s="40"/>
-      <c r="U15" s="38">
+      <c r="T15" s="51"/>
+      <c r="U15" s="49">
         <v>0.8</v>
       </c>
-      <c r="V15" s="40"/>
-      <c r="W15" s="38">
+      <c r="V15" s="51"/>
+      <c r="W15" s="49">
         <v>0.9</v>
       </c>
-      <c r="X15" s="40"/>
+      <c r="X15" s="51"/>
     </row>
     <row r="16" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D16" s="8"/>
       <c r="E16" s="27"/>
       <c r="F16" s="9"/>
-      <c r="G16" s="41" t="s">
+      <c r="G16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="H16" s="42"/>
-      <c r="I16" s="41" t="s">
+      <c r="H16" s="33"/>
+      <c r="I16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="J16" s="42"/>
-      <c r="K16" s="41" t="s">
+      <c r="J16" s="33"/>
+      <c r="K16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="L16" s="51"/>
-      <c r="M16" s="41" t="s">
+      <c r="L16" s="42"/>
+      <c r="M16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="N16" s="42"/>
-      <c r="O16" s="41" t="s">
+      <c r="N16" s="33"/>
+      <c r="O16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="41" t="s">
+      <c r="P16" s="33"/>
+      <c r="Q16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="R16" s="42"/>
-      <c r="S16" s="41" t="s">
+      <c r="R16" s="33"/>
+      <c r="S16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="T16" s="42"/>
-      <c r="U16" s="43" t="s">
+      <c r="T16" s="33"/>
+      <c r="U16" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="V16" s="44"/>
-      <c r="W16" s="43" t="s">
+      <c r="V16" s="35"/>
+      <c r="W16" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="X16" s="44"/>
+      <c r="X16" s="35"/>
     </row>
     <row r="17" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D17" s="10"/>
@@ -3729,14 +3729,14 @@
       </c>
     </row>
     <row r="18" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="45" t="s">
+      <c r="D18" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="48">
+      <c r="E18" s="39">
         <v>0.3</v>
       </c>
       <c r="F18" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G18" s="15">
         <v>1.2</v>
@@ -3794,10 +3794,10 @@
       </c>
     </row>
     <row r="19" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="46"/>
-      <c r="E19" s="49"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="40"/>
       <c r="F19" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G19" s="17">
         <v>15.6</v>
@@ -3855,10 +3855,10 @@
       </c>
     </row>
     <row r="20" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D20" s="46"/>
-      <c r="E20" s="50"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="41"/>
       <c r="F20" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G20" s="21">
         <v>29.167000000000002</v>
@@ -3916,12 +3916,12 @@
       </c>
     </row>
     <row r="21" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D21" s="46"/>
-      <c r="E21" s="48">
+      <c r="D21" s="37"/>
+      <c r="E21" s="39">
         <v>0.6</v>
       </c>
       <c r="F21" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G21" s="30">
         <v>1.2</v>
@@ -3979,10 +3979,10 @@
       </c>
     </row>
     <row r="22" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D22" s="46"/>
-      <c r="E22" s="49"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="40"/>
       <c r="F22" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G22" s="30">
         <v>15.6</v>
@@ -4040,10 +4040,10 @@
       </c>
     </row>
     <row r="23" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="46"/>
-      <c r="E23" s="50"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="41"/>
       <c r="F23" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G23" s="31">
         <v>31.292000000000002</v>
@@ -4101,12 +4101,12 @@
       </c>
     </row>
     <row r="24" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D24" s="46"/>
-      <c r="E24" s="48">
+      <c r="D24" s="37"/>
+      <c r="E24" s="39">
         <v>0.9</v>
       </c>
       <c r="F24" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G24" s="30">
         <v>1.2</v>
@@ -4164,10 +4164,10 @@
       </c>
     </row>
     <row r="25" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D25" s="46"/>
-      <c r="E25" s="49"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="40"/>
       <c r="F25" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G25" s="30">
         <v>15.6</v>
@@ -4225,10 +4225,10 @@
       </c>
     </row>
     <row r="26" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D26" s="47"/>
-      <c r="E26" s="50"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="41"/>
       <c r="F26" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G26" s="31">
         <v>33.119</v>
@@ -4287,16 +4287,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="G13:X14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="S15:T15"/>
-    <mergeCell ref="U15:V15"/>
     <mergeCell ref="D18:D26"/>
     <mergeCell ref="E18:E20"/>
     <mergeCell ref="E21:E23"/>
@@ -4311,6 +4301,16 @@
     <mergeCell ref="S16:T16"/>
     <mergeCell ref="U16:V16"/>
     <mergeCell ref="W16:X16"/>
+    <mergeCell ref="G13:X14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="S15:T15"/>
+    <mergeCell ref="U15:V15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4323,130 +4323,130 @@
   <sheetData>
     <row r="12" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="4:24" x14ac:dyDescent="0.2">
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="H13" s="33"/>
-      <c r="I13" s="33"/>
-      <c r="J13" s="33"/>
-      <c r="K13" s="33"/>
-      <c r="L13" s="33"/>
-      <c r="M13" s="33"/>
-      <c r="N13" s="33"/>
-      <c r="O13" s="33"/>
-      <c r="P13" s="33"/>
-      <c r="Q13" s="33"/>
-      <c r="R13" s="33"/>
-      <c r="S13" s="33"/>
-      <c r="T13" s="33"/>
-      <c r="U13" s="33"/>
-      <c r="V13" s="33"/>
-      <c r="W13" s="33"/>
-      <c r="X13" s="34"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="44"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="44"/>
+      <c r="R13" s="44"/>
+      <c r="S13" s="44"/>
+      <c r="T13" s="44"/>
+      <c r="U13" s="44"/>
+      <c r="V13" s="44"/>
+      <c r="W13" s="44"/>
+      <c r="X13" s="45"/>
     </row>
     <row r="14" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="G14" s="35"/>
-      <c r="H14" s="36"/>
-      <c r="I14" s="36"/>
-      <c r="J14" s="36"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="36"/>
-      <c r="O14" s="36"/>
-      <c r="P14" s="36"/>
-      <c r="Q14" s="36"/>
-      <c r="R14" s="36"/>
-      <c r="S14" s="36"/>
-      <c r="T14" s="36"/>
-      <c r="U14" s="36"/>
-      <c r="V14" s="36"/>
-      <c r="W14" s="36"/>
-      <c r="X14" s="37"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="47"/>
+      <c r="L14" s="47"/>
+      <c r="M14" s="47"/>
+      <c r="N14" s="47"/>
+      <c r="O14" s="47"/>
+      <c r="P14" s="47"/>
+      <c r="Q14" s="47"/>
+      <c r="R14" s="47"/>
+      <c r="S14" s="47"/>
+      <c r="T14" s="47"/>
+      <c r="U14" s="47"/>
+      <c r="V14" s="47"/>
+      <c r="W14" s="47"/>
+      <c r="X14" s="48"/>
     </row>
     <row r="15" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="E15" s="39"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="38">
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="49">
         <v>0.1</v>
       </c>
-      <c r="H15" s="40"/>
-      <c r="I15" s="38">
+      <c r="H15" s="51"/>
+      <c r="I15" s="49">
         <v>0.2</v>
       </c>
-      <c r="J15" s="40"/>
-      <c r="K15" s="38">
+      <c r="J15" s="51"/>
+      <c r="K15" s="49">
         <v>0.3</v>
       </c>
-      <c r="L15" s="40"/>
-      <c r="M15" s="38">
+      <c r="L15" s="51"/>
+      <c r="M15" s="49">
         <v>0.4</v>
       </c>
-      <c r="N15" s="40"/>
-      <c r="O15" s="38">
+      <c r="N15" s="51"/>
+      <c r="O15" s="49">
         <v>0.5</v>
       </c>
-      <c r="P15" s="40"/>
-      <c r="Q15" s="38">
+      <c r="P15" s="51"/>
+      <c r="Q15" s="49">
         <v>0.6</v>
       </c>
-      <c r="R15" s="40"/>
-      <c r="S15" s="38">
+      <c r="R15" s="51"/>
+      <c r="S15" s="49">
         <v>0.7</v>
       </c>
-      <c r="T15" s="40"/>
-      <c r="U15" s="38">
+      <c r="T15" s="51"/>
+      <c r="U15" s="49">
         <v>0.8</v>
       </c>
-      <c r="V15" s="40"/>
-      <c r="W15" s="38">
+      <c r="V15" s="51"/>
+      <c r="W15" s="49">
         <v>0.9</v>
       </c>
-      <c r="X15" s="40"/>
+      <c r="X15" s="51"/>
     </row>
     <row r="16" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D16" s="8"/>
       <c r="E16" s="27"/>
       <c r="F16" s="9"/>
-      <c r="G16" s="41" t="s">
+      <c r="G16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="H16" s="42"/>
-      <c r="I16" s="41" t="s">
+      <c r="H16" s="33"/>
+      <c r="I16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="J16" s="42"/>
-      <c r="K16" s="41" t="s">
+      <c r="J16" s="33"/>
+      <c r="K16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="L16" s="51"/>
-      <c r="M16" s="41" t="s">
+      <c r="L16" s="42"/>
+      <c r="M16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="N16" s="42"/>
-      <c r="O16" s="41" t="s">
+      <c r="N16" s="33"/>
+      <c r="O16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="41" t="s">
+      <c r="P16" s="33"/>
+      <c r="Q16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="R16" s="42"/>
-      <c r="S16" s="41" t="s">
+      <c r="R16" s="33"/>
+      <c r="S16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="T16" s="42"/>
-      <c r="U16" s="43" t="s">
+      <c r="T16" s="33"/>
+      <c r="U16" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="V16" s="44"/>
-      <c r="W16" s="43" t="s">
+      <c r="V16" s="35"/>
+      <c r="W16" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="X16" s="44"/>
+      <c r="X16" s="35"/>
     </row>
     <row r="17" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D17" s="10"/>
@@ -4508,14 +4508,14 @@
       </c>
     </row>
     <row r="18" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="45" t="s">
+      <c r="D18" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="48">
+      <c r="E18" s="39">
         <v>0.3</v>
       </c>
       <c r="F18" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G18" s="15">
         <v>0</v>
@@ -4573,10 +4573,10 @@
       </c>
     </row>
     <row r="19" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="46"/>
-      <c r="E19" s="49"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="40"/>
       <c r="F19" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G19" s="17">
         <v>13.6</v>
@@ -4634,10 +4634,10 @@
       </c>
     </row>
     <row r="20" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D20" s="46"/>
-      <c r="E20" s="50"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="41"/>
       <c r="F20" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G20" s="21">
         <v>41.886000000000003</v>
@@ -4695,12 +4695,12 @@
       </c>
     </row>
     <row r="21" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D21" s="46"/>
-      <c r="E21" s="48">
+      <c r="D21" s="37"/>
+      <c r="E21" s="39">
         <v>0.6</v>
       </c>
       <c r="F21" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G21" s="30">
         <v>0</v>
@@ -4758,10 +4758,10 @@
       </c>
     </row>
     <row r="22" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D22" s="46"/>
-      <c r="E22" s="49"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="40"/>
       <c r="F22" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G22" s="30">
         <v>13.6</v>
@@ -4819,10 +4819,10 @@
       </c>
     </row>
     <row r="23" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="46"/>
-      <c r="E23" s="50"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="41"/>
       <c r="F23" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G23" s="31">
         <v>49.122</v>
@@ -4880,12 +4880,12 @@
       </c>
     </row>
     <row r="24" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D24" s="46"/>
-      <c r="E24" s="48">
+      <c r="D24" s="37"/>
+      <c r="E24" s="39">
         <v>0.9</v>
       </c>
       <c r="F24" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G24" s="30">
         <v>0</v>
@@ -4943,10 +4943,10 @@
       </c>
     </row>
     <row r="25" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D25" s="46"/>
-      <c r="E25" s="49"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="40"/>
       <c r="F25" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G25" s="30">
         <v>14</v>
@@ -5004,10 +5004,10 @@
       </c>
     </row>
     <row r="26" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D26" s="47"/>
-      <c r="E26" s="50"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="41"/>
       <c r="F26" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G26" s="31">
         <v>56.313000000000002</v>
@@ -5066,16 +5066,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="G13:X14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="S15:T15"/>
-    <mergeCell ref="U15:V15"/>
     <mergeCell ref="D18:D26"/>
     <mergeCell ref="E18:E20"/>
     <mergeCell ref="E21:E23"/>
@@ -5090,6 +5080,16 @@
     <mergeCell ref="S16:T16"/>
     <mergeCell ref="U16:V16"/>
     <mergeCell ref="W16:X16"/>
+    <mergeCell ref="G13:X14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="S15:T15"/>
+    <mergeCell ref="U15:V15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5102,130 +5102,130 @@
   <sheetData>
     <row r="12" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="4:24" x14ac:dyDescent="0.2">
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="H13" s="33"/>
-      <c r="I13" s="33"/>
-      <c r="J13" s="33"/>
-      <c r="K13" s="33"/>
-      <c r="L13" s="33"/>
-      <c r="M13" s="33"/>
-      <c r="N13" s="33"/>
-      <c r="O13" s="33"/>
-      <c r="P13" s="33"/>
-      <c r="Q13" s="33"/>
-      <c r="R13" s="33"/>
-      <c r="S13" s="33"/>
-      <c r="T13" s="33"/>
-      <c r="U13" s="33"/>
-      <c r="V13" s="33"/>
-      <c r="W13" s="33"/>
-      <c r="X13" s="34"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="44"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="44"/>
+      <c r="R13" s="44"/>
+      <c r="S13" s="44"/>
+      <c r="T13" s="44"/>
+      <c r="U13" s="44"/>
+      <c r="V13" s="44"/>
+      <c r="W13" s="44"/>
+      <c r="X13" s="45"/>
     </row>
     <row r="14" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="G14" s="35"/>
-      <c r="H14" s="36"/>
-      <c r="I14" s="36"/>
-      <c r="J14" s="36"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="36"/>
-      <c r="O14" s="36"/>
-      <c r="P14" s="36"/>
-      <c r="Q14" s="36"/>
-      <c r="R14" s="36"/>
-      <c r="S14" s="36"/>
-      <c r="T14" s="36"/>
-      <c r="U14" s="36"/>
-      <c r="V14" s="36"/>
-      <c r="W14" s="36"/>
-      <c r="X14" s="37"/>
+      <c r="G14" s="46"/>
+      <c r="H14" s="47"/>
+      <c r="I14" s="47"/>
+      <c r="J14" s="47"/>
+      <c r="K14" s="47"/>
+      <c r="L14" s="47"/>
+      <c r="M14" s="47"/>
+      <c r="N14" s="47"/>
+      <c r="O14" s="47"/>
+      <c r="P14" s="47"/>
+      <c r="Q14" s="47"/>
+      <c r="R14" s="47"/>
+      <c r="S14" s="47"/>
+      <c r="T14" s="47"/>
+      <c r="U14" s="47"/>
+      <c r="V14" s="47"/>
+      <c r="W14" s="47"/>
+      <c r="X14" s="48"/>
     </row>
     <row r="15" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="E15" s="39"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="38">
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="49">
         <v>0.1</v>
       </c>
-      <c r="H15" s="40"/>
-      <c r="I15" s="38">
+      <c r="H15" s="51"/>
+      <c r="I15" s="49">
         <v>0.2</v>
       </c>
-      <c r="J15" s="40"/>
-      <c r="K15" s="38">
+      <c r="J15" s="51"/>
+      <c r="K15" s="49">
         <v>0.3</v>
       </c>
-      <c r="L15" s="40"/>
-      <c r="M15" s="38">
+      <c r="L15" s="51"/>
+      <c r="M15" s="49">
         <v>0.4</v>
       </c>
-      <c r="N15" s="40"/>
-      <c r="O15" s="38">
+      <c r="N15" s="51"/>
+      <c r="O15" s="49">
         <v>0.5</v>
       </c>
-      <c r="P15" s="40"/>
-      <c r="Q15" s="38">
+      <c r="P15" s="51"/>
+      <c r="Q15" s="49">
         <v>0.6</v>
       </c>
-      <c r="R15" s="40"/>
-      <c r="S15" s="38">
+      <c r="R15" s="51"/>
+      <c r="S15" s="49">
         <v>0.7</v>
       </c>
-      <c r="T15" s="40"/>
-      <c r="U15" s="38">
+      <c r="T15" s="51"/>
+      <c r="U15" s="49">
         <v>0.8</v>
       </c>
-      <c r="V15" s="40"/>
-      <c r="W15" s="38">
+      <c r="V15" s="51"/>
+      <c r="W15" s="49">
         <v>0.9</v>
       </c>
-      <c r="X15" s="40"/>
+      <c r="X15" s="51"/>
     </row>
     <row r="16" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D16" s="8"/>
       <c r="E16" s="27"/>
       <c r="F16" s="9"/>
-      <c r="G16" s="41" t="s">
+      <c r="G16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="H16" s="42"/>
-      <c r="I16" s="41" t="s">
+      <c r="H16" s="33"/>
+      <c r="I16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="J16" s="42"/>
-      <c r="K16" s="41" t="s">
+      <c r="J16" s="33"/>
+      <c r="K16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="L16" s="51"/>
-      <c r="M16" s="41" t="s">
+      <c r="L16" s="42"/>
+      <c r="M16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="N16" s="42"/>
-      <c r="O16" s="41" t="s">
+      <c r="N16" s="33"/>
+      <c r="O16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="P16" s="42"/>
-      <c r="Q16" s="41" t="s">
+      <c r="P16" s="33"/>
+      <c r="Q16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="R16" s="42"/>
-      <c r="S16" s="41" t="s">
+      <c r="R16" s="33"/>
+      <c r="S16" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="T16" s="42"/>
-      <c r="U16" s="43" t="s">
+      <c r="T16" s="33"/>
+      <c r="U16" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="V16" s="44"/>
-      <c r="W16" s="43" t="s">
+      <c r="V16" s="35"/>
+      <c r="W16" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="X16" s="44"/>
+      <c r="X16" s="35"/>
     </row>
     <row r="17" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D17" s="10"/>
@@ -5287,14 +5287,14 @@
       </c>
     </row>
     <row r="18" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="45" t="s">
+      <c r="D18" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="48">
+      <c r="E18" s="39">
         <v>0.3</v>
       </c>
       <c r="F18" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G18" s="15">
         <v>1.4</v>
@@ -5352,10 +5352,10 @@
       </c>
     </row>
     <row r="19" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="46"/>
-      <c r="E19" s="49"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="40"/>
       <c r="F19" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G19" s="17">
         <v>21.6</v>
@@ -5413,10 +5413,10 @@
       </c>
     </row>
     <row r="20" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D20" s="46"/>
-      <c r="E20" s="50"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="41"/>
       <c r="F20" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G20" s="21">
         <v>22.558</v>
@@ -5474,12 +5474,12 @@
       </c>
     </row>
     <row r="21" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D21" s="46"/>
-      <c r="E21" s="48">
+      <c r="D21" s="37"/>
+      <c r="E21" s="39">
         <v>0.6</v>
       </c>
       <c r="F21" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G21" s="30">
         <v>1.4</v>
@@ -5537,10 +5537,10 @@
       </c>
     </row>
     <row r="22" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D22" s="46"/>
-      <c r="E22" s="49"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="40"/>
       <c r="F22" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G22" s="30">
         <v>21.6</v>
@@ -5598,10 +5598,10 @@
       </c>
     </row>
     <row r="23" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="46"/>
-      <c r="E23" s="50"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="41"/>
       <c r="F23" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G23" s="31">
         <v>23.004000000000001</v>
@@ -5659,12 +5659,12 @@
       </c>
     </row>
     <row r="24" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D24" s="46"/>
-      <c r="E24" s="48">
+      <c r="D24" s="37"/>
+      <c r="E24" s="39">
         <v>0.9</v>
       </c>
       <c r="F24" s="29" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G24" s="30">
         <v>1.4</v>
@@ -5722,10 +5722,10 @@
       </c>
     </row>
     <row r="25" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D25" s="46"/>
-      <c r="E25" s="49"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="40"/>
       <c r="F25" s="29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G25" s="30">
         <v>21.6</v>
@@ -5783,10 +5783,10 @@
       </c>
     </row>
     <row r="26" spans="4:24" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D26" s="47"/>
-      <c r="E26" s="50"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="41"/>
       <c r="F26" s="29" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G26" s="31">
         <v>23.44</v>
@@ -5845,16 +5845,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="G13:X14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="S15:T15"/>
-    <mergeCell ref="U15:V15"/>
     <mergeCell ref="D18:D26"/>
     <mergeCell ref="E18:E20"/>
     <mergeCell ref="E21:E23"/>
@@ -5869,6 +5859,16 @@
     <mergeCell ref="S16:T16"/>
     <mergeCell ref="U16:V16"/>
     <mergeCell ref="W16:X16"/>
+    <mergeCell ref="G13:X14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="S15:T15"/>
+    <mergeCell ref="U15:V15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>